<commit_message>
CP1: rodada real da sintética fim a fim + relatório; consertos achados pela rodada (encoding do console, path do kit, logs por sessão no ship); célula de fórmula na fixture e template_map mostrando fórmulas
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/unidade_sintetica/template.xlsx
+++ b/tests/fixtures/unidade_sintetica/template.xlsx
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -573,6 +573,17 @@
         <is>
           <t>SURVEY</t>
         </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>TOTAL ACRES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="E2">
+        <f>SUM(B2:B99)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>